<commit_message>
*2 inspections, not 1
</commit_message>
<xml_diff>
--- a/chinatown-chinese-oct2026/unweighted_peak_counts_excel.xlsx
+++ b/chinatown-chinese-oct2026/unweighted_peak_counts_excel.xlsx
@@ -616,11 +616,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="59749863"/>
-        <c:axId val="61881016"/>
+        <c:axId val="42316010"/>
+        <c:axId val="19720737"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="59749863"/>
+        <c:axId val="42316010"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -672,12 +672,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61881016"/>
+        <c:crossAx val="19720737"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="61881016"/>
+        <c:axId val="19720737"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -729,7 +729,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59749863"/>
+        <c:crossAx val="42316010"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2024,7 +2024,7 @@
         <v>67</v>
       </c>
       <c r="D29" s="0" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>45741</v>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="D30" s="0" t="n">
         <f aca="false">AVERAGE(D2:D29)</f>
-        <v>2.39285714285714</v>
+        <v>2.42857142857143</v>
       </c>
       <c r="F30" s="0" t="n">
         <f aca="false">AVERAGE(F2:F29)</f>

</xml_diff>